<commit_message>
Allow for multi-select + comments
</commit_message>
<xml_diff>
--- a/BvA.xlsx
+++ b/BvA.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="10">
   <si>
     <t>Department</t>
   </si>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -451,13 +451,13 @@
         <v>100000</v>
       </c>
       <c r="F2">
-        <v>40000</v>
+        <v>60000</v>
       </c>
       <c r="G2">
-        <v>60000</v>
+        <v>40000</v>
       </c>
       <c r="H2">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -471,13 +471,13 @@
         <v>100000</v>
       </c>
       <c r="F3">
-        <v>40000</v>
+        <v>60001</v>
       </c>
       <c r="G3">
-        <v>20000</v>
+        <v>-20001</v>
       </c>
       <c r="H3">
-        <v>0.4</v>
+        <v>0.60001</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -491,13 +491,13 @@
         <v>100000</v>
       </c>
       <c r="F4">
-        <v>40000</v>
+        <v>60002</v>
       </c>
       <c r="G4">
-        <v>-20000</v>
+        <v>-80003</v>
       </c>
       <c r="H4">
-        <v>0.4</v>
+        <v>0.60002</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -511,13 +511,13 @@
         <v>100000</v>
       </c>
       <c r="F5">
-        <v>40000</v>
+        <v>60003</v>
       </c>
       <c r="G5">
-        <v>-60000</v>
+        <v>-140006</v>
       </c>
       <c r="H5">
-        <v>0.4</v>
+        <v>0.60003</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -531,13 +531,13 @@
         <v>100000</v>
       </c>
       <c r="F6">
-        <v>40000</v>
+        <v>60004</v>
       </c>
       <c r="G6">
-        <v>-100000</v>
+        <v>-200010</v>
       </c>
       <c r="H6">
-        <v>0.4</v>
+        <v>0.60004</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -551,13 +551,13 @@
         <v>100000</v>
       </c>
       <c r="F7">
-        <v>40000</v>
+        <v>60005</v>
       </c>
       <c r="G7">
-        <v>-140000</v>
+        <v>-260015</v>
       </c>
       <c r="H7">
-        <v>0.4</v>
+        <v>0.60005</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -571,13 +571,13 @@
         <v>100000</v>
       </c>
       <c r="F8">
-        <v>40000</v>
+        <v>60006</v>
       </c>
       <c r="G8">
-        <v>-180000</v>
+        <v>-320021</v>
       </c>
       <c r="H8">
-        <v>0.4</v>
+        <v>0.60006</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -591,13 +591,13 @@
         <v>100000</v>
       </c>
       <c r="F9">
-        <v>40000</v>
+        <v>60007</v>
       </c>
       <c r="G9">
-        <v>-220000</v>
+        <v>-380028</v>
       </c>
       <c r="H9">
-        <v>0.4</v>
+        <v>0.60007</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -611,13 +611,13 @@
         <v>100000</v>
       </c>
       <c r="F10">
-        <v>40000</v>
+        <v>60008</v>
       </c>
       <c r="G10">
-        <v>-260000</v>
+        <v>-440036</v>
       </c>
       <c r="H10">
-        <v>0.4</v>
+        <v>0.6000799999999999</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -631,12 +631,212 @@
         <v>100000</v>
       </c>
       <c r="F11">
-        <v>40000</v>
+        <v>60009</v>
       </c>
       <c r="G11">
-        <v>-300000</v>
+        <v>-500045</v>
       </c>
       <c r="H11">
+        <v>0.60009</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12">
+        <v>100000</v>
+      </c>
+      <c r="F12">
+        <v>40000</v>
+      </c>
+      <c r="G12">
+        <v>-540045</v>
+      </c>
+      <c r="H12">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13">
+        <v>100000</v>
+      </c>
+      <c r="F13">
+        <v>40000</v>
+      </c>
+      <c r="G13">
+        <v>-580045</v>
+      </c>
+      <c r="H13">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14">
+        <v>100000</v>
+      </c>
+      <c r="F14">
+        <v>40000</v>
+      </c>
+      <c r="G14">
+        <v>-620045</v>
+      </c>
+      <c r="H14">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15">
+        <v>100000</v>
+      </c>
+      <c r="F15">
+        <v>40000</v>
+      </c>
+      <c r="G15">
+        <v>-660045</v>
+      </c>
+      <c r="H15">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16">
+        <v>100000</v>
+      </c>
+      <c r="F16">
+        <v>40000</v>
+      </c>
+      <c r="G16">
+        <v>-700045</v>
+      </c>
+      <c r="H16">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="17" spans="3:8">
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17">
+        <v>100000</v>
+      </c>
+      <c r="F17">
+        <v>40000</v>
+      </c>
+      <c r="G17">
+        <v>-740045</v>
+      </c>
+      <c r="H17">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="18" spans="3:8">
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18">
+        <v>100000</v>
+      </c>
+      <c r="F18">
+        <v>40000</v>
+      </c>
+      <c r="G18">
+        <v>-780045</v>
+      </c>
+      <c r="H18">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="19" spans="3:8">
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19">
+        <v>100000</v>
+      </c>
+      <c r="F19">
+        <v>40000</v>
+      </c>
+      <c r="G19">
+        <v>-820045</v>
+      </c>
+      <c r="H19">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="20" spans="3:8">
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20">
+        <v>100000</v>
+      </c>
+      <c r="F20">
+        <v>40000</v>
+      </c>
+      <c r="G20">
+        <v>-860045</v>
+      </c>
+      <c r="H20">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="21" spans="3:8">
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21">
+        <v>100000</v>
+      </c>
+      <c r="F21">
+        <v>40000</v>
+      </c>
+      <c r="G21">
+        <v>-900045</v>
+      </c>
+      <c r="H21">
         <v>0.4</v>
       </c>
     </row>
@@ -696,13 +896,13 @@
         <v>100000</v>
       </c>
       <c r="F2">
-        <v>400000</v>
+        <v>1000045</v>
       </c>
       <c r="G2">
-        <v>-300000</v>
+        <v>-900045</v>
       </c>
       <c r="H2">
-        <v>4</v>
+        <v>10.00045</v>
       </c>
     </row>
   </sheetData>

</xml_diff>